<commit_message>
fix(genome): update connector compliance status and my-genome page
</commit_message>
<xml_diff>
--- a/docs/CONNECTOR_COMPLIANCE_STATUS_2026-08-16.xlsx
+++ b/docs/CONNECTOR_COMPLIANCE_STATUS_2026-08-16.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\denni\PycharmProjects\Kira\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{775DB354-D570-4C7F-BE16-554D56D0A9F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9561703-D284-4D19-AA79-DA8F1E6D556A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1234" uniqueCount="713">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1233" uniqueCount="715">
   <si>
     <t>CASA readiness — Kira / Google app</t>
   </si>
@@ -2173,6 +2173,12 @@
   </si>
   <si>
     <t>PresenceGraph</t>
+  </si>
+  <si>
+    <t>artem.gavrilov@dfuture.co</t>
+  </si>
+  <si>
+    <t>Artem</t>
   </si>
 </sst>
 </file>
@@ -4257,39 +4263,46 @@
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="B3" s="11" t="s">
-        <v>613</v>
+      <c r="A3" s="9" t="s">
+        <v>596</v>
+      </c>
+      <c r="B3" s="13" t="s">
+        <v>636</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>623</v>
+        <v>633</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>634</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>653</v>
+        <v>632</v>
       </c>
       <c r="F3" s="9" t="s">
-        <v>630</v>
-      </c>
-      <c r="G3" s="10"/>
-      <c r="H3" s="10"/>
+        <v>635</v>
+      </c>
+      <c r="H3" s="9">
+        <v>1</v>
+      </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" s="9" t="s">
         <v>596</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>636</v>
+        <v>642</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>633</v>
+        <v>643</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>634</v>
+        <v>644</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>632</v>
+        <v>615</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>635</v>
+        <v>645</v>
       </c>
       <c r="H4" s="9">
         <v>1</v>
@@ -4299,20 +4312,17 @@
       <c r="A5" s="9" t="s">
         <v>596</v>
       </c>
-      <c r="B5" s="13" t="s">
-        <v>642</v>
+      <c r="B5" s="9" t="s">
+        <v>605</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>643</v>
-      </c>
-      <c r="D5" s="9" t="s">
-        <v>644</v>
+        <v>629</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>615</v>
+        <v>653</v>
       </c>
       <c r="F5" s="9" t="s">
-        <v>645</v>
+        <v>630</v>
       </c>
       <c r="H5" s="9">
         <v>1</v>
@@ -4322,14 +4332,23 @@
       <c r="A6" s="9" t="s">
         <v>596</v>
       </c>
-      <c r="B6" s="13" t="s">
-        <v>662</v>
+      <c r="B6" s="9" t="s">
+        <v>606</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>663</v>
+        <v>56</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>664</v>
+        <v>627</v>
+      </c>
+      <c r="E6" s="9" t="s">
+        <v>653</v>
+      </c>
+      <c r="F6" s="9" t="s">
+        <v>640</v>
+      </c>
+      <c r="G6" s="9">
+        <v>61402612471</v>
       </c>
       <c r="H6" s="9">
         <v>1</v>
@@ -4339,14 +4358,23 @@
       <c r="A7" s="9" t="s">
         <v>596</v>
       </c>
-      <c r="B7" s="13" t="s">
-        <v>667</v>
+      <c r="B7" s="9" t="s">
+        <v>607</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>668</v>
+        <v>56</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>703</v>
+        <v>628</v>
+      </c>
+      <c r="E7" s="9" t="s">
+        <v>653</v>
+      </c>
+      <c r="F7" s="9" t="s">
+        <v>639</v>
+      </c>
+      <c r="G7" s="9">
+        <v>61402612471</v>
       </c>
       <c r="H7" s="9">
         <v>1</v>
@@ -4356,14 +4384,20 @@
       <c r="A8" s="9" t="s">
         <v>596</v>
       </c>
-      <c r="B8" s="12" t="s">
-        <v>671</v>
+      <c r="B8" s="9" t="s">
+        <v>608</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>672</v>
+        <v>618</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>701</v>
+        <v>619</v>
+      </c>
+      <c r="E8" s="9" t="s">
+        <v>654</v>
+      </c>
+      <c r="F8" s="9" t="s">
+        <v>638</v>
       </c>
       <c r="H8" s="9">
         <v>1</v>
@@ -4374,13 +4408,22 @@
         <v>596</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>681</v>
+        <v>609</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>682</v>
+        <v>56</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>683</v>
+        <v>620</v>
+      </c>
+      <c r="E9" s="9" t="s">
+        <v>653</v>
+      </c>
+      <c r="F9" s="9" t="s">
+        <v>637</v>
+      </c>
+      <c r="G9" s="9">
+        <v>61402612471</v>
       </c>
       <c r="H9" s="9">
         <v>1</v>
@@ -4390,14 +4433,23 @@
       <c r="A10" s="9" t="s">
         <v>596</v>
       </c>
-      <c r="B10" s="13" t="s">
-        <v>687</v>
+      <c r="B10" s="9" t="s">
+        <v>610</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>682</v>
+        <v>621</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>688</v>
+        <v>624</v>
+      </c>
+      <c r="E10" s="9" t="s">
+        <v>655</v>
+      </c>
+      <c r="F10" s="9" t="s">
+        <v>637</v>
+      </c>
+      <c r="G10" s="9">
+        <v>60163034307</v>
       </c>
       <c r="H10" s="9">
         <v>1</v>
@@ -4408,10 +4460,13 @@
         <v>596</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>605</v>
+        <v>611</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>629</v>
+        <v>622</v>
+      </c>
+      <c r="D11" s="9" t="s">
+        <v>625</v>
       </c>
       <c r="E11" s="9" t="s">
         <v>653</v>
@@ -4428,22 +4483,19 @@
         <v>596</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>606</v>
+        <v>612</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>56</v>
+        <v>625</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="E12" s="9" t="s">
         <v>653</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>640</v>
-      </c>
-      <c r="G12" s="9">
-        <v>61402612471</v>
+        <v>631</v>
       </c>
       <c r="H12" s="9">
         <v>1</v>
@@ -4454,22 +4506,16 @@
         <v>596</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>607</v>
+        <v>613</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>56</v>
-      </c>
-      <c r="D13" s="9" t="s">
-        <v>628</v>
+        <v>623</v>
       </c>
       <c r="E13" s="9" t="s">
         <v>653</v>
       </c>
       <c r="F13" s="9" t="s">
-        <v>639</v>
-      </c>
-      <c r="G13" s="9">
-        <v>61402612471</v>
+        <v>630</v>
       </c>
       <c r="H13" s="9">
         <v>1</v>
@@ -4479,20 +4525,11 @@
       <c r="A14" s="9" t="s">
         <v>596</v>
       </c>
-      <c r="B14" s="9" t="s">
-        <v>608</v>
+      <c r="B14" s="11" t="s">
+        <v>713</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>618</v>
-      </c>
-      <c r="D14" s="9" t="s">
-        <v>619</v>
-      </c>
-      <c r="E14" s="9" t="s">
-        <v>654</v>
-      </c>
-      <c r="F14" s="9" t="s">
-        <v>638</v>
+        <v>714</v>
       </c>
       <c r="H14" s="9">
         <v>1</v>
@@ -4502,138 +4539,117 @@
       <c r="A15" s="9" t="s">
         <v>596</v>
       </c>
-      <c r="B15" s="9" t="s">
-        <v>609</v>
+      <c r="B15" s="13" t="s">
+        <v>662</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>56</v>
+        <v>663</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>620</v>
-      </c>
-      <c r="E15" s="9" t="s">
-        <v>653</v>
-      </c>
-      <c r="F15" s="9" t="s">
-        <v>637</v>
-      </c>
-      <c r="G15" s="9">
-        <v>61402612471</v>
+        <v>664</v>
       </c>
       <c r="H15" s="9">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" s="9" t="s">
         <v>596</v>
       </c>
-      <c r="B16" s="9" t="s">
-        <v>610</v>
+      <c r="B16" s="13" t="s">
+        <v>650</v>
       </c>
       <c r="C16" s="9" t="s">
-        <v>621</v>
+        <v>646</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>624</v>
+        <v>647</v>
       </c>
       <c r="E16" s="9" t="s">
-        <v>655</v>
+        <v>652</v>
       </c>
       <c r="F16" s="9" t="s">
-        <v>637</v>
-      </c>
-      <c r="G16" s="9">
-        <v>60163034307</v>
+        <v>709</v>
       </c>
       <c r="H16" s="9">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A17" s="9" t="s">
         <v>596</v>
       </c>
-      <c r="B17" s="9" t="s">
-        <v>611</v>
+      <c r="B17" s="13" t="s">
+        <v>651</v>
       </c>
       <c r="C17" s="9" t="s">
-        <v>622</v>
+        <v>648</v>
       </c>
       <c r="D17" s="9" t="s">
-        <v>625</v>
+        <v>649</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="F17" s="9" t="s">
-        <v>630</v>
+        <v>709</v>
       </c>
       <c r="H17" s="9">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A18" s="9" t="s">
         <v>596</v>
       </c>
-      <c r="B18" s="9" t="s">
-        <v>612</v>
+      <c r="B18" s="13" t="s">
+        <v>659</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>625</v>
+        <v>656</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>626</v>
-      </c>
-      <c r="E18" s="9" t="s">
-        <v>653</v>
+        <v>660</v>
       </c>
       <c r="F18" s="9" t="s">
-        <v>631</v>
+        <v>710</v>
       </c>
       <c r="H18" s="9">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A19" s="9" t="s">
         <v>596</v>
       </c>
-      <c r="B19" s="9" t="s">
-        <v>613</v>
+      <c r="B19" s="13" t="s">
+        <v>661</v>
       </c>
       <c r="C19" s="9" t="s">
-        <v>623</v>
-      </c>
-      <c r="E19" s="9" t="s">
-        <v>653</v>
+        <v>657</v>
+      </c>
+      <c r="D19" s="9" t="s">
+        <v>658</v>
       </c>
       <c r="F19" s="9" t="s">
-        <v>630</v>
+        <v>711</v>
       </c>
       <c r="H19" s="9">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A20" s="9" t="s">
         <v>596</v>
       </c>
-      <c r="B20" s="13" t="s">
-        <v>650</v>
+      <c r="B20" s="12" t="s">
+        <v>665</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>646</v>
-      </c>
-      <c r="D20" s="9" t="s">
-        <v>647</v>
-      </c>
-      <c r="E20" s="9" t="s">
-        <v>652</v>
+        <v>670</v>
       </c>
       <c r="F20" s="9" t="s">
-        <v>709</v>
+        <v>712</v>
       </c>
       <c r="H20" s="9">
         <v>2</v>
@@ -4643,20 +4659,17 @@
       <c r="A21" s="9" t="s">
         <v>596</v>
       </c>
-      <c r="B21" s="13" t="s">
-        <v>651</v>
+      <c r="B21" s="12" t="s">
+        <v>666</v>
       </c>
       <c r="C21" s="9" t="s">
-        <v>648</v>
+        <v>669</v>
       </c>
       <c r="D21" s="9" t="s">
-        <v>649</v>
-      </c>
-      <c r="E21" s="9" t="s">
-        <v>652</v>
+        <v>702</v>
       </c>
       <c r="F21" s="9" t="s">
-        <v>709</v>
+        <v>712</v>
       </c>
       <c r="H21" s="9">
         <v>2</v>
@@ -4667,76 +4680,67 @@
         <v>596</v>
       </c>
       <c r="B22" s="13" t="s">
-        <v>659</v>
+        <v>667</v>
       </c>
       <c r="C22" s="9" t="s">
-        <v>656</v>
+        <v>668</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>660</v>
-      </c>
-      <c r="F22" s="9" t="s">
-        <v>710</v>
+        <v>703</v>
       </c>
       <c r="H22" s="9">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A23" s="9" t="s">
         <v>596</v>
       </c>
-      <c r="B23" s="13" t="s">
-        <v>661</v>
+      <c r="B23" s="12" t="s">
+        <v>671</v>
       </c>
       <c r="C23" s="9" t="s">
-        <v>657</v>
+        <v>672</v>
       </c>
       <c r="D23" s="9" t="s">
-        <v>658</v>
-      </c>
-      <c r="F23" s="9" t="s">
-        <v>711</v>
+        <v>701</v>
       </c>
       <c r="H23" s="9">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A24" s="9" t="s">
         <v>596</v>
       </c>
-      <c r="B24" s="12" t="s">
-        <v>665</v>
+      <c r="B24" s="9" t="s">
+        <v>681</v>
       </c>
       <c r="C24" s="9" t="s">
-        <v>670</v>
-      </c>
-      <c r="F24" s="9" t="s">
-        <v>712</v>
+        <v>682</v>
+      </c>
+      <c r="D24" s="9" t="s">
+        <v>683</v>
       </c>
       <c r="H24" s="9">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A25" s="9" t="s">
         <v>596</v>
       </c>
-      <c r="B25" s="12" t="s">
-        <v>666</v>
+      <c r="B25" s="13" t="s">
+        <v>687</v>
       </c>
       <c r="C25" s="9" t="s">
-        <v>669</v>
+        <v>682</v>
       </c>
       <c r="D25" s="9" t="s">
-        <v>702</v>
-      </c>
-      <c r="F25" s="9" t="s">
-        <v>712</v>
+        <v>688</v>
       </c>
       <c r="H25" s="9">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.35">
@@ -4750,7 +4754,7 @@
         <v>673</v>
       </c>
       <c r="H26" s="9">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.35">
@@ -4764,7 +4768,7 @@
         <v>675</v>
       </c>
       <c r="H27" s="9">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.35">
@@ -4781,7 +4785,7 @@
         <v>678</v>
       </c>
       <c r="H28" s="9">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.35">
@@ -4795,7 +4799,7 @@
         <v>680</v>
       </c>
       <c r="H29" s="9">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.35">
@@ -4812,7 +4816,7 @@
         <v>686</v>
       </c>
       <c r="H30" s="9">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.35">
@@ -4829,7 +4833,7 @@
         <v>691</v>
       </c>
       <c r="H31" s="9">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.35">
@@ -4846,7 +4850,7 @@
         <v>694</v>
       </c>
       <c r="H32" s="9">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.35">
@@ -4863,7 +4867,7 @@
         <v>697</v>
       </c>
       <c r="H33" s="9">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.35">
@@ -4880,7 +4884,7 @@
         <v>700</v>
       </c>
       <c r="H34" s="9">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.35">
@@ -4902,31 +4906,34 @@
       <c r="F35" s="9" t="s">
         <v>708</v>
       </c>
+      <c r="H35" s="9">
+        <v>3</v>
+      </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:I34">
-    <sortCondition ref="H2:H34"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I35">
+    <sortCondition ref="H2:H35"/>
   </sortState>
   <hyperlinks>
     <hyperlink ref="B2" r:id="rId1" xr:uid="{BCA16BC5-E72E-417D-8660-4F06F8926D7B}"/>
-    <hyperlink ref="B4" r:id="rId2" xr:uid="{74234682-8E4E-4F83-BC83-62327E314534}"/>
-    <hyperlink ref="B5" r:id="rId3" xr:uid="{66B71609-DD29-4E61-9251-BE37BF7A631C}"/>
-    <hyperlink ref="B20" r:id="rId4" xr:uid="{B98388BE-B5BF-487F-8D09-DC7DCFE89D57}"/>
-    <hyperlink ref="B21" r:id="rId5" xr:uid="{3FAE12F5-4A68-4A24-B7B5-954CB4504B86}"/>
-    <hyperlink ref="B22" r:id="rId6" xr:uid="{C0C91398-3757-41E6-8A9D-FA98DE64C6F7}"/>
-    <hyperlink ref="B23" r:id="rId7" xr:uid="{9941706B-D467-4DE0-938F-3FDBE1EEE58B}"/>
-    <hyperlink ref="B6" r:id="rId8" xr:uid="{1E252B55-F4C5-49B8-A5C9-3D811ECF7AB9}"/>
-    <hyperlink ref="B7" r:id="rId9" xr:uid="{03450AC9-5411-401A-AF8F-C36BDD035577}"/>
+    <hyperlink ref="B3" r:id="rId2" xr:uid="{74234682-8E4E-4F83-BC83-62327E314534}"/>
+    <hyperlink ref="B4" r:id="rId3" xr:uid="{66B71609-DD29-4E61-9251-BE37BF7A631C}"/>
+    <hyperlink ref="B16" r:id="rId4" xr:uid="{B98388BE-B5BF-487F-8D09-DC7DCFE89D57}"/>
+    <hyperlink ref="B17" r:id="rId5" xr:uid="{3FAE12F5-4A68-4A24-B7B5-954CB4504B86}"/>
+    <hyperlink ref="B18" r:id="rId6" xr:uid="{C0C91398-3757-41E6-8A9D-FA98DE64C6F7}"/>
+    <hyperlink ref="B19" r:id="rId7" xr:uid="{9941706B-D467-4DE0-938F-3FDBE1EEE58B}"/>
+    <hyperlink ref="B15" r:id="rId8" xr:uid="{1E252B55-F4C5-49B8-A5C9-3D811ECF7AB9}"/>
+    <hyperlink ref="B22" r:id="rId9" xr:uid="{03450AC9-5411-401A-AF8F-C36BDD035577}"/>
     <hyperlink ref="B27" r:id="rId10" xr:uid="{3086EFCD-DDAF-4169-9A6B-4B2BF6887B69}"/>
     <hyperlink ref="B29" r:id="rId11" xr:uid="{204CC4B9-3830-4B5E-843C-B03505A9F84A}"/>
-    <hyperlink ref="B10" r:id="rId12" xr:uid="{D4F13634-CF18-4754-AAFE-7A050F0E72C1}"/>
+    <hyperlink ref="B25" r:id="rId12" xr:uid="{D4F13634-CF18-4754-AAFE-7A050F0E72C1}"/>
     <hyperlink ref="B31" r:id="rId13" xr:uid="{466EAFA8-2021-4CB7-A4E7-4B899A92CF7F}"/>
     <hyperlink ref="B32" r:id="rId14" xr:uid="{83CB2688-979F-4A92-8E67-225D6733998C}"/>
     <hyperlink ref="B33" r:id="rId15" xr:uid="{608D3191-9D88-4AA9-B0FC-FFEDD36A0926}"/>
     <hyperlink ref="B34" r:id="rId16" xr:uid="{171D2F51-1A92-49AB-BFF3-73A5A99DCD3E}"/>
     <hyperlink ref="B26" r:id="rId17" xr:uid="{70571F44-946E-4257-8969-623C78C1DB34}"/>
     <hyperlink ref="B35" r:id="rId18" xr:uid="{D419F506-DD5E-4456-BC8A-3C590C5C6CD6}"/>
-    <hyperlink ref="B3" r:id="rId19" xr:uid="{748D7CA1-6D0D-413F-A1E0-016F9C46E92E}"/>
+    <hyperlink ref="B14" r:id="rId19" xr:uid="{6ACC1C9E-60AA-49E8-97A7-C20D618F49CF}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId20"/>

</xml_diff>